<commit_message>
Fix BOM: deduplicate multi-unit components (Q2 UMH3N appeared twice)
KiCad multi-unit symbols (e.g. dual transistor in SOT-363) produce
separate symbol_instances entries for each unit with the same Reference.
The BOM parser now deduplicates by RefDes to avoid reporting Q2 twice.
</commit_message>
<xml_diff>
--- a/releases/BOM_SmartKnob_View.xlsx
+++ b/releases/BOM_SmartKnob_View.xlsx
@@ -1072,7 +1072,7 @@
       </c>
       <c r="B19" s="4" t="inlineStr">
         <is>
-          <t>Q2, Q2</t>
+          <t>Q2</t>
         </is>
       </c>
       <c r="C19" s="4" t="inlineStr"/>
@@ -1087,7 +1087,7 @@
         </is>
       </c>
       <c r="F19" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G19" s="4" t="inlineStr">
         <is>

</xml_diff>